<commit_message>
docs(v0.383): remove obsolete card maps and spell workbook
Refresh balance examples and token references against current cards-data.js. Remove only the legacy ID migration sheet from the unit workbook, preserving all nine remaining worksheet XML parts, values, formulas and styles. Game version and runtime/assets remain unchanged. Validation: 152 tests pass; no obsolete document references; workbook preservation checks and artifact inspection pass.
</commit_message>
<xml_diff>
--- a/판타지아레나_유닛목록.xlsx
+++ b/판타지아레나_유닛목록.xlsx
@@ -16,7 +16,6 @@
     <sheet name="암흑" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="삼국" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="코스트" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="ID이동" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'전체'!$A$2:$N$176</definedName>
@@ -9447,212 +9446,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="36" t="inlineStr">
-        <is>
-          <t>빈 ID 채움 (끝 번호 → 빈 번호). 일러스트 파일명도 같이 바꿔야 함</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="25" t="inlineStr">
-        <is>
-          <t>속성</t>
-        </is>
-      </c>
-      <c r="B2" s="25" t="inlineStr">
-        <is>
-          <t>옛 ID</t>
-        </is>
-      </c>
-      <c r="C2" s="25" t="inlineStr">
-        <is>
-          <t>새 ID</t>
-        </is>
-      </c>
-      <c r="D2" s="25" t="inlineStr">
-        <is>
-          <t>이름</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="27" t="inlineStr">
-        <is>
-          <t>대지</t>
-        </is>
-      </c>
-      <c r="B3" s="27" t="inlineStr">
-        <is>
-          <t>e29</t>
-        </is>
-      </c>
-      <c r="C3" s="27" t="inlineStr">
-        <is>
-          <t>e11</t>
-        </is>
-      </c>
-      <c r="D3" s="27" t="inlineStr">
-        <is>
-          <t>숲요정</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="27" t="inlineStr">
-        <is>
-          <t>불</t>
-        </is>
-      </c>
-      <c r="B4" s="27" t="inlineStr">
-        <is>
-          <t>f29</t>
-        </is>
-      </c>
-      <c r="C4" s="27" t="inlineStr">
-        <is>
-          <t>f28</t>
-        </is>
-      </c>
-      <c r="D4" s="27" t="inlineStr">
-        <is>
-          <t>불꽃요정</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="27" t="inlineStr">
-        <is>
-          <t>바람</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>n29</t>
-        </is>
-      </c>
-      <c r="C5" s="27" t="inlineStr">
-        <is>
-          <t>n22</t>
-        </is>
-      </c>
-      <c r="D5" s="27" t="inlineStr">
-        <is>
-          <t>실프</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="27" t="inlineStr">
-        <is>
-          <t>물</t>
-        </is>
-      </c>
-      <c r="B6" s="27" t="inlineStr">
-        <is>
-          <t>a29</t>
-        </is>
-      </c>
-      <c r="C6" s="27" t="inlineStr">
-        <is>
-          <t>a21</t>
-        </is>
-      </c>
-      <c r="D6" s="27" t="inlineStr">
-        <is>
-          <t>물의요정</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="27" t="inlineStr">
-        <is>
-          <t>빛</t>
-        </is>
-      </c>
-      <c r="B7" s="27" t="inlineStr">
-        <is>
-          <t>l30</t>
-        </is>
-      </c>
-      <c r="C7" s="27" t="inlineStr">
-        <is>
-          <t>l17</t>
-        </is>
-      </c>
-      <c r="D7" s="27" t="inlineStr">
-        <is>
-          <t>황월영</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>빛</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>l29</t>
-        </is>
-      </c>
-      <c r="C8" s="27" t="inlineStr">
-        <is>
-          <t>l25</t>
-        </is>
-      </c>
-      <c r="D8" s="27" t="inlineStr">
-        <is>
-          <t>광휘요정</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="27" t="inlineStr">
-        <is>
-          <t>암흑</t>
-        </is>
-      </c>
-      <c r="B9" s="27" t="inlineStr">
-        <is>
-          <t>d29</t>
-        </is>
-      </c>
-      <c r="C9" s="27" t="inlineStr">
-        <is>
-          <t>d19</t>
-        </is>
-      </c>
-      <c r="D9" s="27" t="inlineStr">
-        <is>
-          <t>그림자요정</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>